<commit_message>
Align audit workbook template
</commit_message>
<xml_diff>
--- a/01-akceleratehq-lead-capture-automation/docs/akceleratehq-automation-audit-crm-template.public.xlsx
+++ b/01-akceleratehq-lead-capture-automation/docs/akceleratehq-automation-audit-crm-template.public.xlsx
@@ -436,13 +436,13 @@
     <t>n8n Routing Note</t>
   </si>
   <si>
-    <t>lead_score &gt;= 75 AND budget is $2,000+</t>
+    <t>audit_score &gt;= 75 OR strong budget + urgency + authority</t>
   </si>
   <si>
     <t>Hot</t>
   </si>
   <si>
-    <t>Send WhatsApp, email summary, and book discovery call</t>
+    <t>Create Calendar event, send discovery email, update sheet status</t>
   </si>
   <si>
     <t>Founder</t>
@@ -454,13 +454,13 @@
     <t>Create high-priority task + send owner alert</t>
   </si>
   <si>
-    <t>lead_score 50-74</t>
+    <t>audit_score 45-74 or useful fit needing review</t>
   </si>
   <si>
     <t>Warm</t>
   </si>
   <si>
-    <t>Send personalized audit summary + 2 questions</t>
+    <t>Send owner review alert and qualification questions</t>
   </si>
   <si>
     <t>Founder/Assistant</t>
@@ -469,16 +469,16 @@
     <t>48 hours</t>
   </si>
   <si>
-    <t>Create nurture sequence</t>
+    <t>Create manual review task + qualification email</t>
   </si>
   <si>
-    <t>lead_score 30-49</t>
+    <t>audit_score below 45 or early exploration stage</t>
   </si>
   <si>
     <t>Cold</t>
   </si>
   <si>
-    <t>Send useful audit result + case study</t>
+    <t>Send nurture email with practical next step</t>
   </si>
   <si>
     <t>Assistant</t>
@@ -550,7 +550,7 @@
     <t>SLOT-001</t>
   </si>
   <si>
-    <t>2026-06-28</t>
+    <t>2026-07-09</t>
   </si>
   <si>
     <t>11:00</t>
@@ -577,7 +577,7 @@
     <t>SLOT-003</t>
   </si>
   <si>
-    <t>2026-06-29</t>
+    <t>2026-07-10</t>
   </si>
   <si>
     <t>SLOT-004</t>
@@ -586,7 +586,7 @@
     <t>SLOT-005</t>
   </si>
   <si>
-    <t>2026-06-30</t>
+    <t>2026-07-13</t>
   </si>
   <si>
     <t>SLOT-006</t>
@@ -703,7 +703,7 @@
     <t>Lead qualification overhead</t>
   </si>
   <si>
-    <t>Lead scoring + WhatsApp follow-up</t>
+    <t>AI audit scoring + smart lead routing</t>
   </si>
   <si>
     <t>1-3 months</t>
@@ -766,7 +766,7 @@
     <t>No follow-up yet</t>
   </si>
   <si>
-    <t>Day 1 WhatsApp</t>
+    <t>Day 1 confirmation email</t>
   </si>
   <si>
     <t>Day 3 Email</t>
@@ -781,7 +781,7 @@
     <t>Closed</t>
   </si>
   <si>
-    <t>WhatsApp Status</t>
+    <t>Follow-up Status</t>
   </si>
   <si>
     <t>Not Sent</t>
@@ -1102,7 +1102,7 @@
     <t>Recommended flow</t>
   </si>
   <si>
-    <t>Google Form → linked response sheet → Apps Script column mapper → Audit Leads tab → n8n webhook → AI scoring / WhatsApp / email / CRM updates</t>
+    <t>Google Form or Sheet row -&gt; Audit Leads tab -&gt; n8n trigger -&gt; AI audit scoring -&gt; Gmail/Calendar routing -&gt; sheet status updates</t>
   </si>
   <si>
     <t>Main n8n tab</t>
@@ -1114,7 +1114,7 @@
     <t>Important columns</t>
   </si>
   <si>
-    <t>processed, status, priority, lead_score, lead_temperature, recommended_offer, recommended_workflow, recommended_action, whatsapp_status, proposal_status</t>
+    <t>processed, status, audit_score, lead_category, priority_reason, recommended_offer, recommended_workflow, next_action, call_status, proposal_status, n8n_response</t>
   </si>
   <si>
     <t>How to use</t>

</xml_diff>